<commit_message>
fix(ci): upgrade to Node 22, fix summary reporting with 470 tests, and update all test reports
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Failed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Failed_Test_Cases.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Failed Test Cases (17)</t>
+          <t>Failed Test Cases (20)</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>TC-AUTH-019</t>
+          <t>TC-AUTH-016</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -517,16 +517,16 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Authentication Test Case 019</t>
+          <t>Authentication Test Case 016</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3.415</v>
+        <v>3.864</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TC-AUTH-020</t>
+          <t>TC-AUTH-017</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Authentication Test Case 020</t>
+          <t>Authentication Test Case 017</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4.369</v>
+        <v>3.791</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
@@ -567,17 +567,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>TC-AUTHZ-029</t>
+          <t>TC-AUTH-040</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Authorization Test Case 029</t>
+          <t>Authentication Test Case 040</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4.77</v>
+        <v>0.635</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>TC-AUTHZ-036</t>
+          <t>TC-AUTHZ-023</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Authorization Test Case 036</t>
+          <t>Authorization Test Case 023</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1.231</v>
+        <v>7.819</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
@@ -627,17 +627,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>TC-NAV-004</t>
+          <t>TC-AUTHZ-027</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Navigation Test Case 004</t>
+          <t>Authorization Test Case 027</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.999</v>
+        <v>5.162</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -657,26 +657,26 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>TC-NAV-027</t>
+          <t>TC-AUTHZ-036</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Navigation Test Case 027</t>
+          <t>Authorization Test Case 036</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>3.355</v>
+        <v>4.024</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -687,26 +687,26 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>TC-UI-004</t>
+          <t>TC-NAV-006</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>UI Validation</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>UI Validation Test Case 004</t>
+          <t>Navigation Test Case 006</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>4.166</v>
+        <v>6.389</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>TC-UI-013</t>
+          <t>TC-UI-003</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -727,16 +727,16 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>UI Validation Test Case 013</t>
+          <t>UI Validation Test Case 003</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>6.679</v>
+        <v>4.805</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>TC-UI-025</t>
+          <t>TC-UI-020</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -757,16 +757,16 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>UI Validation Test Case 025</t>
+          <t>UI Validation Test Case 020</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>6.787</v>
+        <v>4.565</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
@@ -777,7 +777,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>TC-UI-047</t>
+          <t>TC-UI-042</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>UI Validation Test Case 047</t>
+          <t>UI Validation Test Case 042</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5.304</v>
+        <v>3.514</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>TC-FORM-018</t>
+          <t>TC-FORM-006</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Forms Test Case 018</t>
+          <t>Forms Test Case 006</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>3.205</v>
+        <v>5.35</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
@@ -837,26 +837,26 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>TC-CRUD-012</t>
+          <t>TC-FORM-036</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Forms</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>CRUD Operations Test Case 012</t>
+          <t>Forms Test Case 036</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3.369</v>
+        <v>2.062</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
@@ -867,26 +867,26 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>TC-INPUT-016</t>
+          <t>TC-FORM-037</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Forms</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Input Validation Test Case 016</t>
+          <t>Forms Test Case 037</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.084</v>
+        <v>0.891</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
@@ -897,17 +897,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>TC-ERR-001</t>
+          <t>TC-INPUT-007</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Error Handling</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Error Handling Test Case 001</t>
+          <t>Input Validation Test Case 007</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.74</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
@@ -927,17 +927,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>TC-RESP-014</t>
+          <t>TC-ERR-005</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Responsive Design</t>
+          <t>Error Handling</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Responsive Design Test Case 014</t>
+          <t>Error Handling Test Case 005</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5.754</v>
+        <v>7.148</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -957,26 +957,26 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>TC-REG-035</t>
+          <t>TC-SESS-005</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Regression Test Case 035</t>
+          <t>Session Management Test Case 005</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>4.417</v>
+        <v>8.207000000000001</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
@@ -987,17 +987,17 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>TC-REG-044</t>
+          <t>TC-SESS-006</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Regression Test Case 044</t>
+          <t>Session Management Test Case 006</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1006,9 +1006,99 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>3.723</v>
+        <v>2.294</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>AssertionError: Element not found — expected condition failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>TC-SESS-011</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Session Management</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Session Management Test Case 011</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>4.161</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>AssertionError: Element not found — expected condition failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TC-ACC-002</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Accessibility Test Case 002</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>1.718</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>AssertionError: Element not found — expected condition failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TC-PERF-008</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Performance Smoke</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Performance Smoke Test Case 008</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>1.164</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>AssertionError: Element not found — expected condition failed</t>
         </is>

</xml_diff>